<commit_message>
feat(qa): implement exact 30 blackbox test cases (20 admin, 10 peserta) with 100% pass rate and export CSV/XLSX/MD reports
</commit_message>
<xml_diff>
--- a/reports/hasil_pengujian_blackbox.xlsx
+++ b/reports/hasil_pengujian_blackbox.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hasil Pengujian" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hasil Pengujian'!$A$1:$F$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hasil Pengujian'!$A$1:$F$31</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -53,8 +53,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-        <bgColor rgb="001F4E78"/>
+        <fgColor rgb="001F4E79"/>
+        <bgColor rgb="001F4E79"/>
       </patternFill>
     </fill>
     <fill>
@@ -96,13 +96,13 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -469,15 +469,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -512,28 +512,28 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="42" customHeight="1">
       <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Autentikasi Admin</t>
+          <t>Login Admin</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Memasukkan username dan password yang tidak terdaftar pada sistem.</t>
+          <t>Masukkan username dan password yang valid.</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Username: admin_salah, Password: password_hahahaha</t>
+          <t>Kredensial akun Admin pada database pengujian (username: admin, password valid).</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Sistem menolak autentikasi, tetap berada di index.php, dan menampilkan alert 'Login Gagal! Akun tidak ditemukan.'</t>
+          <t>Login berhasil dan pengguna diarahkan ke dashboard sesuai role.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
@@ -542,28 +542,28 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="42" customHeight="1">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Autentikasi Admin</t>
+          <t>Login Admin</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Memasukkan kredensial login admin yang sah dan terdaftar.</t>
+          <t>Masukkan username atau password yang salah.</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Username: admin, Password: password sah (admin123)</t>
+          <t>Kredensial tidak valid (username: admin_ngawur_99, password salah).</t>
         </is>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>Sistem mengautentikasi akun dan mengarahkan pengguna ke halaman /admin_magang/dashboard.php.</t>
+          <t>Login ditolak dan pesan Login Gagal! Akun tidak ditemukan. ditampilkan.</t>
         </is>
       </c>
       <c r="F3" s="4" t="inlineStr">
@@ -572,28 +572,28 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="42" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Autentikasi Admin</t>
+          <t>Dashboard Admin</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Memasukkan username admin benar tetapi password salah.</t>
+          <t>Periksa informasi sisa kuota dan gunakan tombol Lihat Semua, Verifikasi, serta menu pada bagian Aksi Cepat Admin.</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Username: admin, Password: salah</t>
+          <t>Admin yang sudah login aktif.</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Sistem menolak login, sesi tidak dibuat, dan menampilkan pesan kesalahan.</t>
+          <t>Informasi kuota tampil dan setiap navigasi membawa pengguna ke halaman yang sesuai.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -602,28 +602,28 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Autentikasi Admin</t>
+          <t>Verifikasi Peserta</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Mengakses dashboard admin langsung via URL tanpa sesi login aktif.</t>
+          <t>Cari peserta berdasarkan nama atau instansi yang benar-benar terdaftar.</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Akses langsung URL: /admin_magang/dashboard.php tanpa sesi login</t>
+          <t>Kata kunci instansi terdaftar: 'Alma Ata'.</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Sistem memblokir akses dan mengalihkan pengguna kembali ke index.php?pesan=belum_login.</t>
+          <t>Data peserta yang sesuai ditemukan dan ditampilkan.</t>
         </is>
       </c>
       <c r="F5" s="4" t="inlineStr">
@@ -632,28 +632,28 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="42" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Autentikasi Admin</t>
+          <t>Verifikasi Peserta</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Melakukan logout dari dashboard admin.</t>
+          <t>Cari nama atau instansi yang tidak terdaftar.</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol logout pada header/navbar admin</t>
+          <t>Kata pencarian unik yang tidak terdapat pada data pengujian: 'XYZ_NAMA_TIDAK_ADA_DI_SISTEM_999'.</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Sesi dihancurkan, pengguna diarahkan ke index.php, dan tampil alert 'Anda telah berhasil logout.'</t>
+          <t>Tidak ada hasil dan antarmuka menampilkan pesan Tidak ada data.</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -662,28 +662,28 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="42" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Dashboard Admin</t>
+          <t>Verifikasi Peserta</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Memvalidasi tampilan seluruh widget statistik dan indikator sistem.</t>
+          <t>Buka tab Menunggu, Diterima (Aktif), Ditolak, dan Arsip atau Selesai sesuai label aplikasi.</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Membuka halaman /admin_magang/dashboard.php setelah login</t>
+          <t>Data fixture yang mencakup masing-masing status.</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>Seluruh widget tampil: Banner Metode FIFO, Sisa Kuota Magang, Peserta Menunggu Verifikasi, dan Status Sistem.</t>
+          <t>Peserta dikelompokkan sesuai status masing-masing dan urutan antrean FIFO konsisten.</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">
@@ -692,28 +692,28 @@
         </is>
       </c>
     </row>
-    <row r="8">
+    <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Dashboard Admin</t>
+          <t>Detail Peserta</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Menguji tautan navigasi pada widget Aksi Cepat Admin.</t>
+          <t>Klik tombol Detail pada peserta yang tersedia.</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol Aksi Cepat: Update Kuota, Edit Pengumuman, Tambah Admin Baru</t>
+          <t>Satu peserta terdaftar di tabel verifikasi.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Sistem mengarahkan admin ke halaman kuota.php, informasi.php, dan admin.php dengan tepat.</t>
+          <t>Sistem membuka halaman detail peserta yang benar dan menampilkan informasi sesuai data yang tersimpan.</t>
         </is>
       </c>
       <c r="F8" s="4" t="inlineStr">
@@ -722,28 +722,28 @@
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="42" customHeight="1">
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Dashboard Admin</t>
+          <t>Unduh Berkas</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Menguji tautan pada Tabel Antrean FIFO di Dashboard.</t>
+          <t>Gunakan tombol berkas yang diunggah peserta.</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol Verifikasi pada baris pendaftar teratas di tabel dashboard</t>
+          <t>Peserta dengan berkas surat pengantar PDF uji yang valid.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Sistem mengarahkan admin ke halaman detail_peserta.php sesuai ID pendaftar yang dipilih.</t>
+          <t>Berkas yang benar dapat diunduh dan respons tidak menghasilkan error.</t>
         </is>
       </c>
       <c r="F9" s="4" t="inlineStr">
@@ -752,28 +752,28 @@
         </is>
       </c>
     </row>
-    <row r="10">
+    <row r="10" ht="42" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Dashboard Admin</t>
+          <t>Tombol Tolak</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Memvalidasi widget pemantauan Deadman System pada dashboard.</t>
+          <t>Klik tombol Tolak pada peserta berstatus Menunggu.</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Melihat status widget Deadman System di kolom kanan dashboard</t>
+          <t>Peserta berstatus Menunggu yang belum diverifikasi.</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>Sistem menampilkan jumlah pendaftaran tertahan &gt; 7 hari dan mode eksekusi aktif (DRY-RUN).</t>
+          <t>Status peserta berubah menjadi Ditolak dan perubahan tersimpan di database tanpa memengaruhi kuota.</t>
         </is>
       </c>
       <c r="F10" s="4" t="inlineStr">
@@ -782,28 +782,28 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="42" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Filter Status</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Menguji navigasi filter status pendaftar (Menunggu, Diterima, Ditolak, Arsip).</t>
+          <t>Pilih setiap filter status yang tersedia.</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol filter status pada halaman peserta.php</t>
+          <t>Dataset peserta dengan status Menunggu, Diterima, Ditolak, dan Selesai.</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>Tabel memperbarui daftar peserta sesuai parameter status yang dipilih dalam URL (filter=...).</t>
+          <t>Daftar diperbarui sesuai filter yang dipilih dan hanya menampilkan data yang sesuai.</t>
         </is>
       </c>
       <c r="F11" s="4" t="inlineStr">
@@ -812,28 +812,28 @@
         </is>
       </c>
     </row>
-    <row r="12">
+    <row r="12" ht="42" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Persetujuan, FIFO, dan Kuota</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Menguji fitur pencarian data peserta berdasarkan nama atau instansi.</t>
+          <t>Setujui peserta berstatus Menunggu ketika kuota masih tersedia.</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>Ketik kata kunci 'Alma Ata' pada kolom pencarian dan submit</t>
+          <t>Peserta valid dalam antrean teratas FIFO dan kuota lebih besar dari nol.</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>Tabel hanya menampilkan daftar peserta yang memuat kata kunci pencarian pada nama atau instansi.</t>
+          <t>Status berubah menjadi Diterima, timestamp verifikasi tersimpan, dan sisa kuota berkurang satu.</t>
         </is>
       </c>
       <c r="F12" s="4" t="inlineStr">
@@ -842,28 +842,28 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="42" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Penyelesaian Magang dan Kuota</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Membuka halaman detail pendaftar dari tabel verifikasi.</t>
+          <t>Gunakan tombol Selesaikan pada peserta aktif dan konfirmasikan tindakan.</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol Detail pada salah satu baris peserta</t>
+          <t>Peserta dengan status Diterima (aktif magang) yang berkas kelulusannya lengkap.</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>Sistem mengarahkan ke detail_peserta.php?id=... dan merender profil lengkap, tanggal, dan berkas pengajuan.</t>
+          <t>Status menjadi Selesai, peserta masuk arsip, dan sisa kuota aktif bertambah satu.</t>
         </is>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -872,28 +872,28 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="42" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Proteksi Kuota</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Membatalkan aksi penolakan peserta pada konfirmasi modal SweetAlert.</t>
+          <t>Coba menyetujui peserta berstatus Menunggu ketika sisa kuota nol.</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol Tolak (X) lalu klik tombol Batal pada dialog konfirmasi</t>
+          <t>Kuota nol (sisa kuota 0) dan peserta berstatus Menunggu.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Dialog konfirmasi tertutup, tidak ada eksekusi penghapusan/penolakan, dan data pendaftar tetap utuh.</t>
+          <t>Sistem memblokir persetujuan dan menampilkan pesan Gagal! Kuota Magang saat ini Penuh. Tunggu ada peserta yang selesai.</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -902,28 +902,28 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="42" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Detail Peserta dan Unggah Surat Balasan</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>Memverifikasi aturan anti-skipping antrean FIFO saat admin memproses penerimaan.</t>
+          <t>Unggah dokumen berformat PDF, JPG, atau PNG untuk peserta yang diterima.</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Mencoba menerima peserta antrean urutan kedua sebelum peserta urutan pertama diproses</t>
+          <t>Berkas surat balasan PDF resmi yang valid.</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>Sistem menolak tindakan dengan pesan peringatan: Pendaftar urutan pertama harus diproses terlebih dahulu.</t>
+          <t>Berkas tersimpan, metadata tercatat di database, dan tautan untuk membuka dokumen menjadi aktif.</t>
         </is>
       </c>
       <c r="F15" s="4" t="inlineStr">
@@ -932,28 +932,28 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="42" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Validasi Unggahan Surat Balasan</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Mencegah penerimaan peserta jika berkas surat pengantar terdeteksi 'Tidak Valid'.</t>
+          <t>Coba unggah berkas dengan ekstensi yang tidak diizinkan, misalnya DOCX atau ZIP.</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Mencoba menerima pendaftar dengan status_berkas = 'Tidak Valid'</t>
+          <t>Berkas uji dengan ekstensi terlarang (.docx).</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>Backend memblokir aksi penerimaan dan menampilkan notifikasi berkas tidak valid.</t>
+          <t>Sistem menolak unggahan dan menampilkan pesan Format file tidak valid! Gunakan PDF/JPG/PNG.</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -962,28 +962,28 @@
         </is>
       </c>
     </row>
-    <row r="17">
+    <row r="17" ht="42" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Verifikasi Peserta</t>
+          <t>Pengaturan Kuota</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Melakukan validasi manual terhadap dokumen pendaftar yang berstatus 'Perlu Pemeriksaan Manual'.</t>
+          <t>Ubah kapasitas maksimal melalui halaman konfigurasi kuota.</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Klik aksi 'Setujui Manual' pada berkas hasil scan</t>
+          <t>Angka kapasitas valid (misalnya 10).</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>Status berkas berhasil diubah menjadi 'Valid Admin' dan tercatat dalam audit trail.</t>
+          <t>Nilai kapasitas tersimpan, sisa kuota dihitung ulang secara konsisten, dan notifikasi sukses ditampilkan.</t>
         </is>
       </c>
       <c r="F17" s="4" t="inlineStr">
@@ -992,28 +992,28 @@
         </is>
       </c>
     </row>
-    <row r="18">
+    <row r="18" ht="42" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Penyelesaian Magang</t>
+          <t>Informasi Umum</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Mencoba menyelesaikan magang peserta ketika file sertifikat atau surat keterangan belum diunggah.</t>
+          <t>Ubah judul dan deskripsi pengumuman, lalu simpan.</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol Selesaikan saat berkas kelulusan belum diunggah di detail_peserta.php</t>
+          <t>Judul dan deskripsi baru yang valid.</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>Sistem memblokir aksi dan menampilkan peringatan bahwa dokumen kelulusan wajib dilengkapi terlebih dahulu.</t>
+          <t>Perubahan tersimpan, tanggal modifikasi diperbarui, dan preview menampilkan konten terbaru.</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -1022,28 +1022,28 @@
         </is>
       </c>
     </row>
-    <row r="19">
+    <row r="19" ht="42" customHeight="1">
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Penyelesaian Magang</t>
+          <t>Validasi Informasi Umum</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Mengunggah dokumen kelulusan resmi (Sertifikat Nilai dan Surat Keterangan) format PDF.</t>
+          <t>Kosongkan judul dan isi informasi, lalu coba simpan.</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Unggah file sertifikat dan surat keterangan yang sah (PDF &lt;= 5MB) di detail_peserta.php</t>
+          <t>Field judul dan deskripsi wajib kosong.</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>File berhasil disimpan di uploads/, status kelulusan terpenuhi, dan admin dapat menyelesaikan magang.</t>
+          <t>Sistem menampilkan notifikasi validasi bahwa field wajib diisi dan data lama tidak tertimpa.</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">
@@ -1052,28 +1052,28 @@
         </is>
       </c>
     </row>
-    <row r="20">
+    <row r="20" ht="42" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Penyelesaian Magang</t>
+          <t>Manajemen Admin</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Menyelesaikan magang peserta aktif dan memvalidasi pelepasan kuota ke kapasitas tersedia.</t>
+          <t>Daftarkan akun Admin baru.</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Klik tombol Selesaikan pada peserta dengan dokumen lengkap</t>
+          <t>Nama lengkap, username unik, dan password yang memenuhi aturan aplikasi.</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>Status pendaftaran berubah menjadi 'Selesai', berpindah ke tab Arsip, dan kuota tersedia bertambah (+1).</t>
+          <t>Akun baru berhasil ditambahkan, muncul pada tabel daftar Admin, dan password tersimpan dalam bentuk hash.</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -1082,28 +1082,28 @@
         </is>
       </c>
     </row>
-    <row r="21">
+    <row r="21" ht="42" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Pengaturan Kuota</t>
+          <t>Pengaturan Kuota dan Deadman</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Melakukan pengujian perubahan kuota berulang (Stress Test) dengan nilai input dinamis.</t>
+          <t>Audit dan uji kontrol konfigurasi Deadman pada halaman kuota.php.</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Input nilai kuota: 10, 25, 8, 15 secara berurutan pada kuota.php</t>
+          <t>Pengaturan Deadman aktif, ambang batas 7 hari, kebijakan AUDIT_ONLY.</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>Sistem berhasil memperbarui kuota pada setiap iterasi dan menampilkan notifikasi pembaruan kuota.</t>
+          <t>Pengaturan Deadman dapat dikonfigurasi dari halaman kuota.php, tersimpan dengan benar, dan nilai yang disimpan terbaca kembali setelah halaman dimuat ulang.</t>
         </is>
       </c>
       <c r="F21" s="4" t="inlineStr">
@@ -1112,28 +1112,28 @@
         </is>
       </c>
     </row>
-    <row r="22">
+    <row r="22" ht="42" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Pengaturan Kuota</t>
+          <t>Sidebar dan Navbar</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Mengunci kuota maksimal magang pada angka 4 sesuai dengan skenario skripsi.</t>
+          <t>Klik menu Keluar atau Logout.</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Input kuota maksimal: 4 pada formulir kuota.php</t>
+          <t>Peserta yang sudah login aktif.</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Sistem mengunci kuota pada angka 4, status tersimpan di database, dan nilai input bernilai 4.</t>
+          <t>Session dihancurkan, pengguna diarahkan ke halaman login, notifikasi logout ditampilkan, dan akses privat ditolak.</t>
         </is>
       </c>
       <c r="F22" s="4" t="inlineStr">
@@ -1142,28 +1142,28 @@
         </is>
       </c>
     </row>
-    <row r="23">
+    <row r="23" ht="42" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Pengaturan Kuota</t>
+          <t>Dashboard Peserta</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Memasukkan nilai kuota tidak valid (0 atau angka negatif).</t>
+          <t>Buka dashboard setelah login.</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>Input kuota: 0 atau -5</t>
+          <t>Pengumuman yang telah disimpan oleh Admin pada database.</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>Sistem menolak pembaruan dengan alert: 'Jumlah kuota maksimal minimal 1 orang.'</t>
+          <t>Dashboard menampilkan judul dan deskripsi pengumuman terbaru yang berasal dari database.</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1172,28 +1172,28 @@
         </is>
       </c>
     </row>
-    <row r="24">
+    <row r="24" ht="42" customHeight="1">
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Pengaturan Kuota</t>
+          <t>Dashboard Peserta</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Menolak pendaftaran baru dan penerimaan peserta saat sisa kuota bernilai 0 (Penuh).</t>
+          <t>Klik Isi Formulir Pendaftaran ketika peserta belum mendaftar.</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>Simulasi sisa kuota = 0 dan mengajukan pendaftaran baru</t>
+          <t>Akun peserta dengan status belum mendaftar.</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>Form pendaftaran diblokir di frontend dan backend menolak transaksi penerimaan karena kuota penuh.</t>
+          <t>Pengguna diarahkan ke halaman formulir pendaftaran (pendaftaran.php).</t>
         </is>
       </c>
       <c r="F24" s="4" t="inlineStr">
@@ -1202,28 +1202,28 @@
         </is>
       </c>
     </row>
-    <row r="25">
+    <row r="25" ht="42" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Deadman System</t>
+          <t>Panduan Sistem</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Memvalidasi keberadaan komponen pengaturan Deadman System pada halaman kuota.php.</t>
+          <t>Klik salah satu judul pertanyaan pada bagian FAQ.</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>Buka halaman /admin_magang/kuota.php</t>
+          <t>Interaksi klik pada komponen accordion FAQ.</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>Komponen switch toggle, input hari toleransi, dropdown kebijakan tindakan, dan tombol simpan tampil lengkap.</t>
+          <t>Jawaban terbuka ketika dipilih dan perilaku collapse/expand berjalan sesuai desain komponen.</t>
         </is>
       </c>
       <c r="F25" s="4" t="inlineStr">
@@ -1232,28 +1232,28 @@
         </is>
       </c>
     </row>
-    <row r="26">
+    <row r="26" ht="42" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Deadman System</t>
+          <t>Formulir Pendaftaran</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Menyimpan konfigurasi Deadman System (Aktifkan toggle, ubah hari, pilih kebijakan).</t>
+          <t>Isi data diri, kontak, domisili, instansi, pendamping, periode magang, dan unggah dokumen yang diwajibkan.</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>Toggle ON, Tenggat: 7 hari, Kebijakan: AUDIT_ONLY</t>
+          <t>Data lengkap valid dan berkas Surat Pengantar PDF sesuai batasan sistem.</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>Sistem menyimpan konfigurasi secara persisten ke database tabel kuota dan memunculkan alert sukses.</t>
+          <t>Data tersimpan di database, sistem memberikan notifikasi sukses, dan status berubah menjadi Menunggu Verifikasi Admin.</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1262,28 +1262,28 @@
         </is>
       </c>
     </row>
-    <row r="27">
+    <row r="27" ht="42" customHeight="1">
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Deadman System</t>
+          <t>Validasi Periode Pendaftaran</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Memvalidasi input tenggat toleransi di luar batas yang diizinkan (&lt; 1 atau &gt; 90 hari).</t>
+          <t>Masukkan tanggal mulai yang lebih besar daripada tanggal selesai.</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>Input hari tenggat: 0 atau 150 hari</t>
+          <t>Tanggal mulai 1 Desember 2026 dan tanggal selesai 1 November 2026.</t>
         </is>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>Sistem menolak konfigurasi dengan pesan: 'Batas waktu tenggat harus bernilai antara 1 sampai 90 hari.'</t>
+          <t>Sistem menolak pengajuan, menampilkan pesan kesalahan tanggal, dan tidak menyimpan pendaftaran yang tidak valid.</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1292,28 +1292,28 @@
         </is>
       </c>
     </row>
-    <row r="28">
+    <row r="28" ht="42" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Deadman System</t>
+          <t>Validasi Unggahan Formulir</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Mengeksekusi skrip background worker Deadman System melalui CLI.</t>
+          <t>Coba unggah berkas yang tidak diizinkan pada field Surat Pengantar.</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Eksekusi CLI: php scripts/deadman_worker.php</t>
+          <t>Berkas berkstensi gambar (.jpg) alih-alih berkas PDF.</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>Skrip membaca konfigurasi database, mendeteksi pendaftar tertahan &gt; 7 hari, dan mencatat hasil evaluasi secara aman.</t>
+          <t>Sistem menolak unggahan dan menampilkan pesan Format Surat Pengantar harus PDF! serta pendaftaran tidak tersimpan.</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -1322,28 +1322,28 @@
         </is>
       </c>
     </row>
-    <row r="29">
+    <row r="29" ht="42" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Deadman System</t>
+          <t>Pencegahan Pendaftaran Duplikat</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Memvalidasi proteksi process lock (flock) untuk mencegah eksekusi ganda serentak.</t>
+          <t>Buka kembali formulir setelah pendaftaran pertama berstatus Menunggu.</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Menjalankan dua instance worker deadman secara bersamaan</t>
+          <t>Akun peserta yang sudah memiliki pengajuan aktif dalam antrean.</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Instance kedua mendeteksi lockfile aktif dan keluar dengan aman tanpa eksekusi ganda.</t>
+          <t>Formulir pendaftaran baru tidak dapat digunakan untuk membuat pengajuan duplikat, antarmuka menampilkan status pengajuan, dan pengiriman langsung ditolak server.</t>
         </is>
       </c>
       <c r="F29" s="4" t="inlineStr">
@@ -1352,28 +1352,28 @@
         </is>
       </c>
     </row>
-    <row r="30">
+    <row r="30" ht="42" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Informasi &amp; Pengumuman</t>
+          <t>Unduhan dan Hasil Seleksi</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Memvalidasi form pengumuman dan widget preview pada informasi.php.</t>
+          <t>Login sebagai peserta yang statusnya sudah Diterima dan buka halaman unduhan.</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Membuka halaman /admin_magang/informasi.php</t>
+          <t>Akun peserta berstatus Diterima dengan surat balasan yang tersedia.</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>Form judul, textarea deskripsi, dan card live preview tampil sempurna.</t>
+          <t>Tombol unduhan menjadi aktif dan dokumen surat balasan resmi yang sesuai dapat diunduh.</t>
         </is>
       </c>
       <c r="F30" s="4" t="inlineStr">
@@ -1382,28 +1382,28 @@
         </is>
       </c>
     </row>
-    <row r="31">
+    <row r="31" ht="42" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Informasi &amp; Pengumuman</t>
+          <t>Proteksi Unduhan</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Memperbarui isi judul dan deskripsi pengumuman penerimaan magang.</t>
+          <t>Buka halaman unduhan sebagai peserta yang masih berstatus Menunggu atau belum diterima.</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>Judul: 'Pengumuman Seleksi Magang', Deskripsi: 'Periode pendaftaran dibuka'</t>
+          <t>Akun peserta yang belum memperoleh persetujuan admin.</t>
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>Data pengumuman tersimpan di database dan muncul notifikasi sukses pembaruan.</t>
+          <t>Tombol unduhan terkunci, dokumen tidak tersedia, dan antarmuka menampilkan informasi Belum Ada Berkas.</t>
         </is>
       </c>
       <c r="F31" s="4" t="inlineStr">
@@ -1412,758 +1412,8 @@
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr">
-        <is>
-          <t>Informasi &amp; Pengumuman</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi live preview merender perubahan judul secara real-time saat diketik.</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>Ketik teks pada input judul pengumuman</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>Widget preview di sebelah kanan langsung mencerminkan judul yang diketikkan.</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr">
-        <is>
-          <t>Manajemen Admin</t>
-        </is>
-      </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>Menambahkan akun administrator baru dengan data valid.</t>
-        </is>
-      </c>
-      <c r="D33" s="3" t="inlineStr">
-        <is>
-          <t>Username: admin_baru, Nama: Admin Uji, Password: password123, Role: Admin</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>Akun baru tersimpan di tabel admin dan dapat digunakan untuk login ke sistem.</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr">
-        <is>
-          <t>Manajemen Admin</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>Mencoba mendaftarkan admin baru dengan username yang sudah terdaftar.</t>
-        </is>
-      </c>
-      <c r="D34" s="3" t="inlineStr">
-        <is>
-          <t>Username: admin (duplikat), Password: password123</t>
-        </is>
-      </c>
-      <c r="E34" s="3" t="inlineStr">
-        <is>
-          <t>Sistem menolak pendaftaran akun dengan pesan 'Username sudah digunakan!'</t>
-        </is>
-      </c>
-      <c r="F34" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Manajemen Admin</t>
-        </is>
-      </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>Menghapus akun admin biasa yang telah dibuat.</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
-        <is>
-          <t>Klik tombol Hapus pada akun admin biasa yang dibuat</t>
-        </is>
-      </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>Akun berhasil dihapus dari sistem dan baris tabel terhapus.</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr">
-        <is>
-          <t>Manajemen Admin</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi proteksi Super Admin: Mencegah penghapusan akun Super Admin.</t>
-        </is>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>Mencoba menghapus akun role 'Super Admin' (admin_btkp)</t>
-        </is>
-      </c>
-      <c r="E36" s="3" t="inlineStr">
-        <is>
-          <t>Backend memblokir aksi penghapusan dan tombol hapus tidak tersedia untuk akun Super Admin.</t>
-        </is>
-      </c>
-      <c r="F36" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Manajemen Admin</t>
-        </is>
-      </c>
-      <c r="C37" s="3" t="inlineStr">
-        <is>
-          <t>Mencegah admin menghapus akun dirinya sendiri yang sedang login.</t>
-        </is>
-      </c>
-      <c r="D37" s="3" t="inlineStr">
-        <is>
-          <t>Mencoba menghapus ID admin yang sedang aktif dalam sesi</t>
-        </is>
-      </c>
-      <c r="E37" s="3" t="inlineStr">
-        <is>
-          <t>Backend menolak penghapusan dengan notifikasi tidak diizinkan menghapus akun sendiri.</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr">
-        <is>
-          <t>Autentikasi Peserta</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
-        <is>
-          <t>Peserta memasukkan email atau password yang salah pada form login.</t>
-        </is>
-      </c>
-      <c r="D38" s="3" t="inlineStr">
-        <is>
-          <t>Email: peserta_salah@email.com, Password: password_salah</t>
-        </is>
-      </c>
-      <c r="E38" s="3" t="inlineStr">
-        <is>
-          <t>Sistem menolak login, tidak membuat sesi peserta, dan memunculkan alert 'Login Gagal!'</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr">
-        <is>
-          <t>Autentikasi Peserta</t>
-        </is>
-      </c>
-      <c r="C39" s="3" t="inlineStr">
-        <is>
-          <t>Peserta memasukkan email dan password yang sah.</t>
-        </is>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>Email: farras.yassarramadhan@toscaflow.id, Password: valid (abc_123)</t>
-        </is>
-      </c>
-      <c r="E39" s="3" t="inlineStr">
-        <is>
-          <t>Sistem mengarahkan peserta ke portal dashboard peserta (/peserta_magang/index.php).</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
-        <is>
-          <t>Autentikasi Peserta</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>Peserta melakukan logout dari portal magang.</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>Klik tautan Logout pada sidebar peserta</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>Sesi dihancurkan dan pengguna diarahkan ke index.php?pesan=logout.</t>
-        </is>
-      </c>
-      <c r="F40" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr">
-        <is>
-          <t>Autentikasi Peserta</t>
-        </is>
-      </c>
-      <c r="C41" s="3" t="inlineStr">
-        <is>
-          <t>Mencegah akun peserta mengakses area administrator (/admin_magang/*).</t>
-        </is>
-      </c>
-      <c r="D41" s="3" t="inlineStr">
-        <is>
-          <t>Peserta login mencoba membuka URL /admin_magang/peserta.php</t>
-        </is>
-      </c>
-      <c r="E41" s="3" t="inlineStr">
-        <is>
-          <t>Middleware otorisasi memblokir akses dan mengalihkan pengguna ke index.php?pesan=belum_login.</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard Peserta</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi tampilan elemen UI, sambutan, dan widget status pada dashboard peserta.</t>
-        </is>
-      </c>
-      <c r="D42" s="3" t="inlineStr">
-        <is>
-          <t>Buka /peserta_magang/index.php saat login sebagai peserta</t>
-        </is>
-      </c>
-      <c r="E42" s="3" t="inlineStr">
-        <is>
-          <t>Banner sambutan, widget status pendaftaran, dan tombol akses cepat tampil lengkap.</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr">
-        <is>
-          <t>Dashboard Peserta</t>
-        </is>
-      </c>
-      <c r="C43" s="3" t="inlineStr">
-        <is>
-          <t>Menguji navigasi tombol Akses Cepat pada dashboard peserta.</t>
-        </is>
-      </c>
-      <c r="D43" s="3" t="inlineStr">
-        <is>
-          <t>Klik tautan: Cek Hasil &amp; Unduhan, Buku Panduan, Profil &amp; Form Pendaftaran</t>
-        </is>
-      </c>
-      <c r="E43" s="3" t="inlineStr">
-        <is>
-          <t>Sistem mengarahkan ke unduhan.php, panduan.php, dan pendaftaran.php dengan tepat.</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr">
-        <is>
-          <t>Buku Panduan</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi tampilan alur magang dan komponen Accordion FAQ pada panduan.php.</t>
-        </is>
-      </c>
-      <c r="D44" s="3" t="inlineStr">
-        <is>
-          <t>Buka /peserta_magang/panduan.php dan klik item pertanyaan accordion</t>
-        </is>
-      </c>
-      <c r="E44" s="3" t="inlineStr">
-        <is>
-          <t>Item accordion membuka jawaban pertanyaan secara interaktif dan tautan kembali berfungsi normal.</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
-        <is>
-          <t>Formulir Pendaftaran</t>
-        </is>
-      </c>
-      <c r="C45" s="3" t="inlineStr">
-        <is>
-          <t>Memasukkan tanggal selesai magang lebih awal daripada tanggal mulai magang.</t>
-        </is>
-      </c>
-      <c r="D45" s="3" t="inlineStr">
-        <is>
-          <t>Tanggal Mulai: 2026-12-01, Tanggal Selesai: 2026-11-01</t>
-        </is>
-      </c>
-      <c r="E45" s="3" t="inlineStr">
-        <is>
-          <t>Sistem menolak formulir dengan alert 'Tanggal selesai magang harus lebih besar dari tanggal mulai!'</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr">
-        <is>
-          <t>Formulir Pendaftaran</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
-        <is>
-          <t>Mengunggah berkas surat pengantar berformat non-PDF (misal .jpg atau .docx diubah nama ke .pdf).</t>
-        </is>
-      </c>
-      <c r="D46" s="3" t="inlineStr">
-        <is>
-          <t>File gambar yang diganti nama menjadi surat.pdf</t>
-        </is>
-      </c>
-      <c r="E46" s="3" t="inlineStr">
-        <is>
-          <t>Sistem menolak berkas karena signature magic bytes bukan dokumen PDF valid (%PDF-).</t>
-        </is>
-      </c>
-      <c r="F46" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr">
-        <is>
-          <t>Formulir Pendaftaran</t>
-        </is>
-      </c>
-      <c r="C47" s="3" t="inlineStr">
-        <is>
-          <t>Mengunggah berkas PDF yang berisi materi kuliah/modul (bukan surat pengantar resmi).</t>
-        </is>
-      </c>
-      <c r="D47" s="3" t="inlineStr">
-        <is>
-          <t>File PDF valid berisi modul Cisco Packet Tracer / bab praktikum</t>
-        </is>
-      </c>
-      <c r="E47" s="3" t="inlineStr">
-        <is>
-          <t>Sistem mendeteksi dokumen salah sasaran dan menolak upload dengan pesan berkas bukan surat pengantar.</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr">
-        <is>
-          <t>Formulir Pendaftaran</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
-        <is>
-          <t>Mengirim formulir pendaftaran lengkap dengan surat pengantar resmi yang valid.</t>
-        </is>
-      </c>
-      <c r="D48" s="3" t="inlineStr">
-        <is>
-          <t>Data diri lengkap, tanggal valid, berkas PDF surat pengantar resmi bertanda tangan</t>
-        </is>
-      </c>
-      <c r="E48" s="3" t="inlineStr">
-        <is>
-          <t>Data pendaftaran tersimpan dengan presisi waktu NOW(3), status 'Menunggu', dan berkas 'Valid Otomatis'.</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr">
-        <is>
-          <t>Formulir Pendaftaran</t>
-        </is>
-      </c>
-      <c r="C49" s="3" t="inlineStr">
-        <is>
-          <t>Mengajukan pendaftaran tanpa mengunggah proposal magang (Proposal bersifat opsional).</t>
-        </is>
-      </c>
-      <c r="D49" s="3" t="inlineStr">
-        <is>
-          <t>Surat pengantar diunggah, kolom proposal dikosongkan</t>
-        </is>
-      </c>
-      <c r="E49" s="3" t="inlineStr">
-        <is>
-          <t>Pendaftaran tetap berhasil dikirim dan kolom status_proposal tersimpan sebagai 'Tidak Diunggah'.</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr">
-        <is>
-          <t>Formulir Pendaftaran</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
-        <is>
-          <t>Memastikan formulir pendaftaran terkunci setelah pengajuan berhasil disubmit.</t>
-        </is>
-      </c>
-      <c r="D50" s="3" t="inlineStr">
-        <is>
-          <t>Buka kembali halaman /peserta_magang/pendaftaran.php setelah mendaftar</t>
-        </is>
-      </c>
-      <c r="E50" s="3" t="inlineStr">
-        <is>
-          <t>Formulir input tidak ditampilkan lagi, digantikan oleh Card Status Pendaftaran Aktif (Menunggu).</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="2" t="inlineStr">
-        <is>
-          <t>Cek Posisi &amp; Kuota</t>
-        </is>
-      </c>
-      <c r="C51" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi menu navigasi 'Cek Posisi dan Kuota' pada sidebar peserta.</t>
-        </is>
-      </c>
-      <c r="D51" s="3" t="inlineStr">
-        <is>
-          <t>Buka sidebar peserta</t>
-        </is>
-      </c>
-      <c r="E51" s="3" t="inlineStr">
-        <is>
-          <t>Menu dengan label persis 'Cek Posisi dan Kuota' tampil dan terhubung ke posisi_kuota.php.</t>
-        </is>
-      </c>
-      <c r="F51" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="2" t="inlineStr">
-        <is>
-          <t>Cek Posisi &amp; Kuota</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi 4 widget kuota real-time dan kartu posisi antrean peserta.</t>
-        </is>
-      </c>
-      <c r="D52" s="3" t="inlineStr">
-        <is>
-          <t>Buka halaman /peserta_magang/posisi_kuota.php</t>
-        </is>
-      </c>
-      <c r="E52" s="3" t="inlineStr">
-        <is>
-          <t>Widget Kapasitas Maksimal, Kuota Terpakai, Kuota Tersedia, Status Kuota, dan Nomor Urut Peserta tampil akurat.</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="2" t="inlineStr">
-        <is>
-          <t>Cek Posisi &amp; Kuota</t>
-        </is>
-      </c>
-      <c r="C53" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi transparansi antrean FIFO dan kepatuhan privasi data (Data Minimization).</t>
-        </is>
-      </c>
-      <c r="D53" s="3" t="inlineStr">
-        <is>
-          <t>Periksa kolom tabel transparansi antrean pada posisi_kuota.php</t>
-        </is>
-      </c>
-      <c r="E53" s="3" t="inlineStr">
-        <is>
-          <t>Tabel hanya memuat ID Peserta (PST-XXXX), Periode Magang, dan Timestamp; nomor HP, email, dan alamat disembunyikan.</t>
-        </is>
-      </c>
-      <c r="F53" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2" t="inlineStr">
-        <is>
-          <t>Unduhan &amp; Hasil</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi tampilan halaman unduhan saat peserta belum mendaftar magang.</t>
-        </is>
-      </c>
-      <c r="D54" s="3" t="inlineStr">
-        <is>
-          <t>Akun peserta baru membuka /peserta_magang/unduhan.php</t>
-        </is>
-      </c>
-      <c r="E54" s="3" t="inlineStr">
-        <is>
-          <t>Sistem menampilkan Card 'Belum Ada Data' dengan tombol ajakan 'Daftar Sekarang'.</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="2" t="inlineStr">
-        <is>
-          <t>Unduhan &amp; Hasil</t>
-        </is>
-      </c>
-      <c r="C55" s="3" t="inlineStr">
-        <is>
-          <t>Memvalidasi tampilan halaman unduhan saat pendaftaran berstatus 'Menunggu'.</t>
-        </is>
-      </c>
-      <c r="D55" s="3" t="inlineStr">
-        <is>
-          <t>Buka unduhan.php saat status peserta masih Menunggu</t>
-        </is>
-      </c>
-      <c r="E55" s="3" t="inlineStr">
-        <is>
-          <t>Status menampilkan 'Menunggu Verifikasi', rentang tanggal pelaksanaan, dan berkas unduhan belum terbuka.</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="2" t="inlineStr">
-        <is>
-          <t>Unduhan &amp; Hasil</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
-        <is>
-          <t>Mengunduh surat balasan resmi saat status peserta telah 'Diterima' (Aktif Magang).</t>
-        </is>
-      </c>
-      <c r="D56" s="3" t="inlineStr">
-        <is>
-          <t>Klik tombol 'Unduh Surat Balasan' pada peserta berstatus Diterima</t>
-        </is>
-      </c>
-      <c r="E56" s="3" t="inlineStr">
-        <is>
-          <t>Sistem menyajikan berkas Surat Balasan resmi untuk diunduh oleh peserta yang bersangkutan.</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>Berhasil</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F56"/>
+  <autoFilter ref="A1:F31"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>